<commit_message>
added google calendar dynamic
</commit_message>
<xml_diff>
--- a/src/backend_lc/job_application_tracker.xlsx
+++ b/src/backend_lc/job_application_tracker.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1023,6 +1023,646 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Fri, 13 Jun 2025 21:04:54 +0000</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>SynergisticIT</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Application Received</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>ZipRecruiter &lt;alerts@ziprecruiter.com&gt;</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Kalyan Raju Keerthipati, SynergisticIT has an open position</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Sat, 14 Jun 2025 05:24:29 +0000</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>plogics</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Application Received</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Indeed &lt;donotreply@match.indeed.com&gt;</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>AI and senior AI Engineer (Artificial Intelligence Engineer - NLP and CV) @ plogics</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Sat, 14 Jun 2025 05:24:29 +0000</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>plogics</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Application Received</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Indeed &lt;donotreply@match.indeed.com&gt;</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>AI and senior AI Engineer (Artificial Intelligence Engineer - NLP and CV) @ plogics</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Sat, 14 Jun 2025 06:26:04 +0000</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>LibertyJobs</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Application Received</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Indeed Apply &lt;indeedapply@indeed.com&gt;</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Indeed Application: Data Analytics Product Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Sat, 14 Jun 2025 06:26:04 +0000</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>LibertyJobs</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Application Received</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Indeed Apply &lt;indeedapply@indeed.com&gt;</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Indeed Application: Data Analytics Product Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Sat, 14 Jun 2025 06:26:04 +0000</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>LibertyJobs</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Application Received</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Indeed Apply &lt;indeedapply@indeed.com&gt;</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Indeed Application: Data Analytics Product Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Sat, 14 Jun 2025 06:26:04 +0000</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>LibertyJobs</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Application Received</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Indeed Apply &lt;indeedapply@indeed.com&gt;</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Indeed Application: Data Analytics Product Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Sat, 14 Jun 2025 06:26:04 +0000</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>LibertyJobs</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Application Received</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Indeed Apply &lt;indeedapply@indeed.com&gt;</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Indeed Application: Data Analytics Product Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Sat, 14 Jun 2025 06:26:04 +0000</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Application Received</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Indeed Apply &lt;indeedapply@indeed.com&gt;</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Indeed Application: Data Analytics Product Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Sat, 14 Jun 2025 06:26:04 +0000</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>LibertyJobs</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Application Received</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Indeed Apply &lt;indeedapply@indeed.com&gt;</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Indeed Application: Data Analytics Product Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Sat, 14 Jun 2025 12:26:03 +0000</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Genpact</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Interview Scheduled</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>"Genpact (Video Call) Interview" &lt;info@skill.getujobs.com&gt;</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Genpact ( Video Call ) Interview TOMORROW.. Your application has been processed</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Sat, 14 Jun 2025 15:35:57 +0000</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>ATC</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Application Received</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>2025-06-04</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Paige Edwards &lt;paige@atc-training.store&gt;</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Re: Kalyan, your next step for the BA role at ATC</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Sat, 14 Jun 2025 15:35:57 +0000</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>ATC</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Online Assessment</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>2025-06-04</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Paige Edwards &lt;paige@atc-training.store&gt;</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Re: Kalyan, your next step for the BA role at ATC</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Sat, 14 Jun 2025 15:35:57 +0000</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>ATC</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Online Assessment</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>2025-06-04</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Paige Edwards &lt;paige@atc-training.store&gt;</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Re: Kalyan, your next step for the BA role at ATC</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Sat, 14 Jun 2025 15:35:57 +0000</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>ATC</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Online Assessment</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>2025-06-04</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Paige Edwards &lt;paige@atc-training.store&gt;</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Re: Kalyan, your next step for the BA role at ATC</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Sat, 14 Jun 2025 15:35:57 +0000</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>ATC</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Online Assessment</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>2025-06-04</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Paige Edwards &lt;paige@atc-training.store&gt;</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Re: Kalyan, your next step for the BA role at ATC</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Sat, 14 Jun 2025 15:35:57 +0000</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>ATC</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Online Assessment</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>2025-06-04</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Paige Edwards &lt;paige@atc-training.store&gt;</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Re: Kalyan, your next step for the BA role at ATC</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Sat, 14 Jun 2025 15:35:57 +0000</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>ATC</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Update / In Progress</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>2025-06-04</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Paige Edwards &lt;paige@atc-training.store&gt;</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Re: Kalyan, your next step for the BA role at ATC</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Sat, 14 Jun 2025 15:35:57 +0000</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>ATC</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Update / In Progress</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>2025-06-04</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Paige Edwards &lt;paige@atc-training.store&gt;</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Re: Kalyan, your next step for the BA role at ATC</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Sat, 14 Jun 2025 19:47:04 +0000</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Application Received</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>no-reply@us.greenhouse-mail.io</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Thank you for applying to Discord!</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>